<commit_message>
IMPROVEMENT-SPEC: stock-out auto-SUMIF from SALES LOG (single entry point), Payment column, GCASH & LOAD ledger sheet, dashboard +GCash fees/Today/MTD cards — 18/18 formula-eval
</commit_message>
<xml_diff>
--- a/NegosyoSheet-Demo.xlsx
+++ b/NegosyoSheet-Demo.xlsx
@@ -13,12 +13,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALES LOG" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UTANG" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXPENSES" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GCASH &amp; LOAD" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'INVENTORY'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'SALES LOG'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'SALES LOG'!$A$1:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'UTANG'!$A$1:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'EXPENSES'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'GCASH &amp; LOAD'!$A$1:$E$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -94,7 +96,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -114,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF7E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E9F9F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +160,9 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -562,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F30"/>
+  <dimension ref="B2:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -623,7 +633,7 @@
       <c r="C8" s="4" t="n"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>NET (profit − expenses) (₱)</t>
+          <t>NET (profit + gcash fees − expenses) (₱)</t>
         </is>
       </c>
       <c r="F8" s="4" t="n"/>
@@ -635,7 +645,7 @@
       </c>
       <c r="C9" s="4" t="n"/>
       <c r="E9" s="5">
-        <f>SUM('SALES LOG'!G2:G6)-SUM(EXPENSES!D2:D6)</f>
+        <f>SUM('SALES LOG'!G2:G6)+SUM('GCASH &amp; LOAD'!D2:D6)-SUM(EXPENSES!D2:D6)</f>
         <v/>
       </c>
       <c r="F9" s="4" t="n"/>
@@ -695,69 +705,110 @@
     <row r="17">
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>TOTAL PER ITEM (sales):</t>
-        </is>
-      </c>
+          <t>GCASH/LOAD KITA (fees)</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n"/>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>TOP BUYERS (utang):</t>
-        </is>
-      </c>
+          <t>BENTA NGAYONG ARAW</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Sales (₱)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="11">
-        <f>IF(INVENTORY!A2="","",INVENTORY!A2)</f>
-        <v/>
-      </c>
-      <c r="C19" s="12">
-        <f>IF(INVENTORY!A2="","",SUMIF('SALES LOG'!B:B,INVENTORY!A2,'SALES LOG'!E:E))</f>
-        <v/>
-      </c>
+      <c r="B18" s="11">
+        <f>SUM('GCASH &amp; LOAD'!D2:D6)</f>
+        <v/>
+      </c>
+      <c r="C18" s="10" t="n"/>
+      <c r="E18" s="11">
+        <f>SUMIF('SALES LOG'!A2:A6,TODAY(),'SALES LOG'!E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F18" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="11">
-        <f>IF(INVENTORY!A3="","",INVENTORY!A3)</f>
-        <v/>
-      </c>
-      <c r="C20" s="12">
-        <f>IF(INVENTORY!A3="","",SUMIF('SALES LOG'!B:B,INVENTORY!A3,'SALES LOG'!E:E))</f>
-        <v/>
-      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>BENTA NGAYONG BUWAN (MTD)</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="11">
+        <f>SUMIFS('SALES LOG'!E2:E6,'SALES LOG'!A2:A6,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'SALES LOG'!A2:A6,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
+        <v/>
+      </c>
+      <c r="C21" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL PER ITEM (sales):</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>TOP BUYERS (utang):</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Sales (₱)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="14">
+        <f>IF(INVENTORY!A2="","",INVENTORY!A2)</f>
+        <v/>
+      </c>
+      <c r="C26" s="15">
+        <f>IF(INVENTORY!A2="","",SUMIF('SALES LOG'!B:B,INVENTORY!A2,'SALES LOG'!E:E))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="14">
+        <f>IF(INVENTORY!A3="","",INVENTORY!A3)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15">
+        <f>IF(INVENTORY!A3="","",SUMIF('SALES LOG'!B:B,INVENTORY!A3,'SALES LOG'!E:E))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="14">
         <f>IF(INVENTORY!A4="","",INVENTORY!A4)</f>
         <v/>
       </c>
-      <c r="C21" s="12">
+      <c r="C28" s="15">
         <f>IF(INVENTORY!A4="","",SUMIF('SALES LOG'!B:B,INVENTORY!A4,'SALES LOG'!E:E))</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="11">
+    <row r="29">
+      <c r="B29" s="14">
         <f>IF(INVENTORY!A5="","",INVENTORY!A5)</f>
         <v/>
       </c>
-      <c r="C22" s="12">
+      <c r="C29" s="15">
         <f>IF(INVENTORY!A5="","",SUMIF('SALES LOG'!B:B,INVENTORY!A5,'SALES LOG'!E:E))</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="13" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>DEMO VERSION — 5 rows lang ang pwede. Full version: unlimited rows + free updates.</t>
         </is>
@@ -774,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B24"/>
+  <dimension ref="B2:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -789,7 +840,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Para sa sari-sari store, online reseller, at maliliit na negosyo</t>
         </is>
@@ -799,28 +850,28 @@
       <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>PAANO GAMITIN (3 steps lang):</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>1. I-fill ang INVENTORY sheet — item name, cost, selling price, stock-in, at reorder point.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>2. I-log ang bawat benta sa SALES LOG (may dropdown na item list, auto-compute ang profit).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>3. I-log ang utang sa UTANG at mga gastos sa EXPENSES. Watch ang DASHBOARD — lahat nandoon.</t>
         </is>
@@ -830,90 +881,104 @@
       <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>MGA SHEET:</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>• DASHBOARD — total sales, profit, inventory value, utang, at reorder alerts. Dito ang summary.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>• INVENTORY — listahan ng items. Auto-compute: current stock, stock value, REORDER NA alert.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>• SALES LOG — bawat sale. Auto: unit price (galing Inventory), total, cost, profit.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>• UTANG — listahan ng mga utang. Auto: days overdue at KULIKAHIN NA! alert.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>• EXPENSES — kuryente, upa, load, at iba. Ibaon sa DASHBOARD computation.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>• GCASH &amp; LOAD — cash-in/out, e-load, bills payment logs + kita sa fees.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>• Stock out ay AUTO na galing SALES LOG — isang log lang, walang doble!</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>IMPORTANTE:</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="16" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>• Wag i-edit ang mga may formula (kulay grey). Type lang sa white cells.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="16" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>• Gumagana sa Excel at Google Sheets (i-upload lang sa Drive → Open with Google Sheets).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="16" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>• Ang profit sa SALES LOG = total benta − cost ng items. Ang NET sa DASHBOARD = profit − expenses.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="17" t="inlineStr">
+    <row r="23">
+      <c r="B23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>NegosyoSheet v1.0 · 2026-08-22 · Support: check README sa page where you downloaded</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="13" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>*** DEMO VERSION — limited to 5 inventory rows. Get the full version para walang limit! ***</t>
         </is>
@@ -946,206 +1011,215 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Item Name</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>Cost (₱)</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>Selling Price (₱)</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="21" t="inlineStr">
         <is>
           <t>Stock In</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
-        <is>
-          <t>Stock Out</t>
-        </is>
-      </c>
-      <c r="G1" s="18" t="inlineStr">
+      <c r="F1" s="21" t="inlineStr">
+        <is>
+          <t>Stock Out (auto)</t>
+        </is>
+      </c>
+      <c r="G1" s="21" t="inlineStr">
         <is>
           <t>Current Stock</t>
         </is>
       </c>
-      <c r="H1" s="18" t="inlineStr">
+      <c r="H1" s="21" t="inlineStr">
         <is>
           <t>Stock Value (₱)</t>
         </is>
       </c>
-      <c r="I1" s="18" t="inlineStr">
+      <c r="I1" s="21" t="inlineStr">
         <is>
           <t>Reorder Point</t>
         </is>
       </c>
-      <c r="J1" s="18" t="inlineStr">
+      <c r="J1" s="21" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Noka Noodles</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>pc</t>
         </is>
       </c>
-      <c r="C2" s="20" t="n">
+      <c r="C2" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="D2" s="20" t="n">
+      <c r="D2" s="23" t="n">
         <v>18</v>
       </c>
-      <c r="E2" s="19" t="n">
+      <c r="E2" s="22" t="n">
         <v>48</v>
       </c>
-      <c r="F2" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" s="19">
+      <c r="F2" s="22">
+        <f>IF(A2="","",SUMIF('SALES LOG'!B:B,A2,'SALES LOG'!C:C))</f>
+        <v/>
+      </c>
+      <c r="G2" s="22">
         <f>IF(A2="","",E2-F2)</f>
         <v/>
       </c>
-      <c r="H2" s="20">
+      <c r="H2" s="23">
         <f>IF(A2="","",G2*C2)</f>
         <v/>
       </c>
-      <c r="I2" s="19" t="n"/>
-      <c r="J2" s="19">
+      <c r="I2" s="22" t="n"/>
+      <c r="J2" s="22">
         <f>IF(A2="","",IF(G2&lt;=I2,"⚠️ REORDER NA!","OK"))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Softdrinks 1L</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>btl</t>
         </is>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="23" t="n">
         <v>68</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="23" t="n">
         <v>90</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="22" t="n">
         <v>24</v>
       </c>
-      <c r="F3" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="19">
+      <c r="F3" s="22">
+        <f>IF(A3="","",SUMIF('SALES LOG'!B:B,A3,'SALES LOG'!C:C))</f>
+        <v/>
+      </c>
+      <c r="G3" s="22">
         <f>IF(A3="","",E3-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="20">
+      <c r="H3" s="23">
         <f>IF(A3="","",G3*C3)</f>
         <v/>
       </c>
-      <c r="I3" s="19" t="n"/>
-      <c r="J3" s="19">
+      <c r="I3" s="22" t="n"/>
+      <c r="J3" s="22">
         <f>IF(A3="","",IF(G3&lt;=I3,"⚠️ REORDER NA!","OK"))</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Sabon 60g</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>pc</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="23" t="n">
         <v>22</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="23" t="n">
         <v>35</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="22" t="n">
         <v>30</v>
       </c>
-      <c r="F4" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="G4" s="19">
+      <c r="F4" s="22">
+        <f>IF(A4="","",SUMIF('SALES LOG'!B:B,A4,'SALES LOG'!C:C))</f>
+        <v/>
+      </c>
+      <c r="G4" s="22">
         <f>IF(A4="","",E4-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="20">
+      <c r="H4" s="23">
         <f>IF(A4="","",G4*C4)</f>
         <v/>
       </c>
-      <c r="I4" s="19" t="n"/>
-      <c r="J4" s="19">
+      <c r="I4" s="22" t="n"/>
+      <c r="J4" s="22">
         <f>IF(A4="","",IF(G4&lt;=I4,"⚠️ REORDER NA!","OK"))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="19" t="n"/>
-      <c r="G5" s="19">
+      <c r="A5" s="22" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22">
+        <f>IF(A5="","",SUMIF('SALES LOG'!B:B,A5,'SALES LOG'!C:C))</f>
+        <v/>
+      </c>
+      <c r="G5" s="22">
         <f>IF(A5="","",E5-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="23">
         <f>IF(A5="","",G5*C5)</f>
         <v/>
       </c>
-      <c r="I5" s="19" t="n"/>
-      <c r="J5" s="19">
+      <c r="I5" s="22" t="n"/>
+      <c r="J5" s="22">
         <f>IF(A5="","",IF(G5&lt;=I5,"⚠️ REORDER NA!","OK"))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
-      <c r="G6" s="19">
+      <c r="A6" s="22" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22">
+        <f>IF(A6="","",SUMIF('SALES LOG'!B:B,A6,'SALES LOG'!C:C))</f>
+        <v/>
+      </c>
+      <c r="G6" s="22">
         <f>IF(A6="","",E6-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="23">
         <f>IF(A6="","",G6*C6)</f>
         <v/>
       </c>
-      <c r="I6" s="19" t="n"/>
-      <c r="J6" s="19">
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="22">
         <f>IF(A6="","",IF(G6&lt;=I6,"⚠️ REORDER NA!","OK"))</f>
         <v/>
       </c>
@@ -1170,7 +1244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1180,180 +1254,194 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Item Name</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>Unit Price (₱)</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="21" t="inlineStr">
         <is>
           <t>Total (₱)</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
+      <c r="F1" s="21" t="inlineStr">
         <is>
           <t>Cost (₱)</t>
         </is>
       </c>
-      <c r="G1" s="18" t="inlineStr">
+      <c r="G1" s="21" t="inlineStr">
         <is>
           <t>Profit (₱)</t>
         </is>
       </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Noka Noodles</t>
         </is>
       </c>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="23">
         <f>IF(OR(B2="",C2=""),"",IFERROR(VLOOKUP(B2,INVENTORY!A:D,4,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E2" s="20">
+      <c r="E2" s="23">
         <f>IF(OR(B2="",C2=""),"",D2*C2)</f>
         <v/>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="23">
         <f>IF(OR(B2="",C2=""),"",IFERROR(VLOOKUP(B2,INVENTORY!A:C,3,FALSE),"")*C2)</f>
         <v/>
       </c>
-      <c r="G2" s="20">
+      <c r="G2" s="23">
         <f>IF(OR(B2="",C2=""),"",E2-F2)</f>
         <v/>
       </c>
+      <c r="H2" s="22" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Softdrinks 1L</t>
         </is>
       </c>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="23">
         <f>IF(OR(B3="",C3=""),"",IFERROR(VLOOKUP(B3,INVENTORY!A:D,4,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E3" s="20">
+      <c r="E3" s="23">
         <f>IF(OR(B3="",C3=""),"",D3*C3)</f>
         <v/>
       </c>
-      <c r="F3" s="20">
+      <c r="F3" s="23">
         <f>IF(OR(B3="",C3=""),"",IFERROR(VLOOKUP(B3,INVENTORY!A:C,3,FALSE),"")*C3)</f>
         <v/>
       </c>
-      <c r="G3" s="20">
+      <c r="G3" s="23">
         <f>IF(OR(B3="",C3=""),"",E3-F3)</f>
         <v/>
       </c>
+      <c r="H3" s="22" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="n"/>
-      <c r="B4" s="19" t="n"/>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="20">
+      <c r="A4" s="24" t="n"/>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="23">
         <f>IF(OR(B4="",C4=""),"",IFERROR(VLOOKUP(B4,INVENTORY!A:D,4,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E4" s="20">
+      <c r="E4" s="23">
         <f>IF(OR(B4="",C4=""),"",D4*C4)</f>
         <v/>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="23">
         <f>IF(OR(B4="",C4=""),"",IFERROR(VLOOKUP(B4,INVENTORY!A:C,3,FALSE),"")*C4)</f>
         <v/>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="23">
         <f>IF(OR(B4="",C4=""),"",E4-F4)</f>
         <v/>
       </c>
+      <c r="H4" s="22" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="20">
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="23">
         <f>IF(OR(B5="",C5=""),"",IFERROR(VLOOKUP(B5,INVENTORY!A:D,4,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E5" s="20">
+      <c r="E5" s="23">
         <f>IF(OR(B5="",C5=""),"",D5*C5)</f>
         <v/>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="23">
         <f>IF(OR(B5="",C5=""),"",IFERROR(VLOOKUP(B5,INVENTORY!A:C,3,FALSE),"")*C5)</f>
         <v/>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="23">
         <f>IF(OR(B5="",C5=""),"",E5-F5)</f>
         <v/>
       </c>
+      <c r="H5" s="22" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="n"/>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="20">
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="23">
         <f>IF(OR(B6="",C6=""),"",IFERROR(VLOOKUP(B6,INVENTORY!A:D,4,FALSE),""))</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="23">
         <f>IF(OR(B6="",C6=""),"",D6*C6)</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="23">
         <f>IF(OR(B6="",C6=""),"",IFERROR(VLOOKUP(B6,INVENTORY!A:C,3,FALSE),"")*C6)</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="23">
         <f>IF(OR(B6="",C6=""),"",E6-F6)</f>
         <v/>
       </c>
+      <c r="H6" s="22" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:H6"/>
   <conditionalFormatting sqref="G2:G6">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=INVENTORY!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Cash,GCash,Utang"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1380,123 +1468,123 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>Item / Notes</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>Amount (₱)</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="21" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
+      <c r="F1" s="21" t="inlineStr">
         <is>
           <t>Paid?</t>
         </is>
       </c>
-      <c r="G1" s="18" t="inlineStr">
+      <c r="G1" s="21" t="inlineStr">
         <is>
           <t>Days Overdue</t>
         </is>
       </c>
-      <c r="H1" s="18" t="inlineStr">
+      <c r="H1" s="21" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="n"/>
-      <c r="B2" s="19" t="n"/>
-      <c r="C2" s="19" t="n"/>
-      <c r="D2" s="20" t="n"/>
-      <c r="E2" s="21" t="n"/>
-      <c r="F2" s="19" t="n"/>
-      <c r="G2" s="19">
+      <c r="A2" s="24" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="24" t="n"/>
+      <c r="F2" s="22" t="n"/>
+      <c r="G2" s="22">
         <f>IF(OR(E2="",F2="Yes"),"",MAX(0,TODAY()-E2))</f>
         <v/>
       </c>
-      <c r="H2" s="19">
+      <c r="H2" s="22">
         <f>IF(F2="Yes","✅ PAID",IF(A2="","",IF(G2&gt;0,"🔴 KULIKAHIN NA!","🕒 Hindi pa due")))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="n"/>
-      <c r="B3" s="19" t="n"/>
-      <c r="C3" s="19" t="n"/>
-      <c r="D3" s="20" t="n"/>
-      <c r="E3" s="21" t="n"/>
-      <c r="F3" s="19" t="n"/>
-      <c r="G3" s="19">
+      <c r="A3" s="24" t="n"/>
+      <c r="B3" s="22" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="24" t="n"/>
+      <c r="F3" s="22" t="n"/>
+      <c r="G3" s="22">
         <f>IF(OR(E3="",F3="Yes"),"",MAX(0,TODAY()-E3))</f>
         <v/>
       </c>
-      <c r="H3" s="19">
+      <c r="H3" s="22">
         <f>IF(F3="Yes","✅ PAID",IF(A3="","",IF(G3&gt;0,"🔴 KULIKAHIN NA!","🕒 Hindi pa due")))</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="n"/>
-      <c r="B4" s="19" t="n"/>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="20" t="n"/>
-      <c r="E4" s="21" t="n"/>
-      <c r="F4" s="19" t="n"/>
-      <c r="G4" s="19">
+      <c r="A4" s="24" t="n"/>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="23" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="22">
         <f>IF(OR(E4="",F4="Yes"),"",MAX(0,TODAY()-E4))</f>
         <v/>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="22">
         <f>IF(F4="Yes","✅ PAID",IF(A4="","",IF(G4&gt;0,"🔴 KULIKAHIN NA!","🕒 Hindi pa due")))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="21" t="n"/>
-      <c r="F5" s="19" t="n"/>
-      <c r="G5" s="19">
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="22">
         <f>IF(OR(E5="",F5="Yes"),"",MAX(0,TODAY()-E5))</f>
         <v/>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="22">
         <f>IF(F5="Yes","✅ PAID",IF(A5="","",IF(G5&gt;0,"🔴 KULIKAHIN NA!","🕒 Hindi pa due")))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="n"/>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="21" t="n"/>
-      <c r="F6" s="19" t="n"/>
-      <c r="G6" s="19">
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="22">
         <f>IF(OR(E6="",F6="Yes"),"",MAX(0,TODAY()-E6))</f>
         <v/>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="22">
         <f>IF(F6="Yes","✅ PAID",IF(A6="","",IF(G6&gt;0,"🔴 KULIKAHIN NA!","🕒 Hindi pa due")))</f>
         <v/>
       </c>
@@ -1533,56 +1621,56 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>Amount (₱)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="n"/>
-      <c r="B2" s="19" t="n"/>
-      <c r="C2" s="19" t="n"/>
-      <c r="D2" s="20" t="n"/>
+      <c r="A2" s="24" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="23" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="n"/>
-      <c r="B3" s="19" t="n"/>
-      <c r="C3" s="19" t="n"/>
-      <c r="D3" s="20" t="n"/>
+      <c r="A3" s="24" t="n"/>
+      <c r="B3" s="22" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="23" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="n"/>
-      <c r="B4" s="19" t="n"/>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="20" t="n"/>
+      <c r="A4" s="24" t="n"/>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="23" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="20" t="n"/>
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="23" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="n"/>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="20" t="n"/>
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="23" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D6"/>
@@ -1593,4 +1681,93 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>Amount (₱)</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>Fee Collected (₱)</t>
+        </is>
+      </c>
+      <c r="E1" s="21" t="inlineStr">
+        <is>
+          <t>Customer / Ref No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="24" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="23" t="n"/>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="22" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="n"/>
+      <c r="B3" s="22" t="n"/>
+      <c r="C3" s="23" t="n"/>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="22" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="n"/>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="23" t="n"/>
+      <c r="D4" s="23" t="n"/>
+      <c r="E4" s="22" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="22" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="22" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E6"/>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Cash-In,Cash-Out,E-Load,Bills Payment"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>